<commit_message>
docs(examples): add chart type examples (area, bar, column, pie, scatter, etc.)
12 chart types with py/md/xlsx triplets for AI-friendly learning.
</commit_message>
<xml_diff>
--- a/examples/excel/charts-line.xlsx
+++ b/examples/excel/charts-line.xlsx
@@ -3,13 +3,13 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="R07348e2e24d64303"/>
-    <x:sheet name="2-Line Styles" sheetId="3" r:id="Rabcd157a92f14e19"/>
-    <x:sheet name="3-Line Variants" sheetId="4" r:id="Rb3d2e0be611240a6"/>
-    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="R6b7b79b4bb164d73"/>
-    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="R56a36020a7474f56"/>
-    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="R273f7a256bca4711"/>
-    <x:sheet name="7-Line Elements" sheetId="8" r:id="Ra8030ba92ed44110"/>
+    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="Rbfd0efb35aec4963"/>
+    <x:sheet name="2-Line Styles" sheetId="3" r:id="R9dcb3ba848624399"/>
+    <x:sheet name="3-Line Variants" sheetId="4" r:id="R8e58dc1bf99b49d4"/>
+    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="Rc4ed387a26d64175"/>
+    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="R1419b94eba1c4d69"/>
+    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="R4d6786efd93548e6"/>
+    <x:sheet name="7-Line Elements" sheetId="8" r:id="R9f86d56a43334d3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4553,7 +4553,6 @@
           </c:val>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="1"/>
           <c:showCatName val="0"/>
@@ -9998,7 +9997,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1fd8747d48444509"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R82829a5de6ca470e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10028,7 +10027,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R007e3221a060425a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ac388eaeaf44e10"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10058,7 +10057,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b99792e48be49a2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R100cf27edf564e83"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10088,7 +10087,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf10a6b62b4a24424"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R03c89398da534425"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10123,7 +10122,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6755e941f12f49ce"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e7fc478db724364"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10153,7 +10152,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3bf6cb00e5b4b37"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R841ee3ecb7d0402e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10183,7 +10182,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7e38e17f4664949"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red44bd9154c24230"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10213,7 +10212,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7d49f0a17b0d4998"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fd2c4af072545ff"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10248,7 +10247,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R31c30e7a8cdf4805"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R021cd8f727964d61"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10278,7 +10277,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R601ce7b4dc134810"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf4b57813c5db4e19"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10308,7 +10307,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9c0c8d6c6084516"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra1612f53fb1e4161"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10338,7 +10337,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfcaeada6b1df49c1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re94ae6bf33f4466a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10373,7 +10372,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd6e9204353744be4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R75aad71dea244387"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10403,7 +10402,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2d00411f3efd4909"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fa09b1ea30548bd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10433,7 +10432,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6f5720cc581941e3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a1a02607934c97"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10463,7 +10462,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R861b813cd1cc4723"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R949f5b039fb34a51"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10498,7 +10497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b29e578179c49b6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06b22162442e48b6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10528,7 +10527,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0668b0d28b3342a5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabd58a4f2a184bad"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10558,7 +10557,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R947afb5fce0945f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48ef8511e5a44b87"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10588,7 +10587,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfb205428431240d9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0276fa5e078a45a5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10623,7 +10622,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R601242dccd104580"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52d8ffb89eb74f4c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10653,7 +10652,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc90a430567ef47dd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc598170c9d43401b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10683,7 +10682,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rffef394309804500"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85863529710a43c3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10713,7 +10712,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b9aa3f427414484"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0254af189de4690"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10748,7 +10747,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bf0b077149849c3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R84ee8024b2924161"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10778,7 +10777,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c434f2524e54303"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R46f87f3b69aa4bf4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10808,7 +10807,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d98715520cf450b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d936f56f57142d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10838,7 +10837,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf055a04a9d846d4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcd02a2c4cccc44b4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -11078,48 +11077,48 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba62104c01a547ba"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16f2ef06580438c"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08bdcc4aa67440b2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R622d87bf24db424a"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c73af1674cf4ab5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R274a82bc11674dff"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b9e9a9c891403d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb2c7f1920614886"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccfd96f4b4b34a8c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727c62ff98bc43b9"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0fdeb125d27413d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfee2e49219574a0b"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff87f1e5018a4768"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf044d4fd7a4014"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(examples): regenerate charts-line.xlsx demo file
</commit_message>
<xml_diff>
--- a/examples/excel/charts-line.xlsx
+++ b/examples/excel/charts-line.xlsx
@@ -3,13 +3,13 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="Rbfd0efb35aec4963"/>
-    <x:sheet name="2-Line Styles" sheetId="3" r:id="R9dcb3ba848624399"/>
-    <x:sheet name="3-Line Variants" sheetId="4" r:id="R8e58dc1bf99b49d4"/>
-    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="Rc4ed387a26d64175"/>
-    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="R1419b94eba1c4d69"/>
-    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="R4d6786efd93548e6"/>
-    <x:sheet name="7-Line Elements" sheetId="8" r:id="R9f86d56a43334d3b"/>
+    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="R24c97b32ff404052"/>
+    <x:sheet name="2-Line Styles" sheetId="3" r:id="Rd4cc8124281e4f94"/>
+    <x:sheet name="3-Line Variants" sheetId="4" r:id="R179dea0c8282414f"/>
+    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="R3b0ab19ce75042dd"/>
+    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="R9f13b691275b40be"/>
+    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="Rab7a8a2eb6af40ed"/>
+    <x:sheet name="7-Line Elements" sheetId="8" r:id="R98d15ac20ad94cd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:style val="3"/>
   <c:chart>
     <c:title>
@@ -1321,7 +1321,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -1809,7 +1809,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2361,7 +2361,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2720,7 +2720,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2971,7 +2971,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3130,7 +3130,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3322,7 +3322,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3823,7 +3823,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3946,7 +3946,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -4458,7 +4458,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -4747,7 +4747,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart22.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5112,7 +5112,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart23.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5350,7 +5350,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart24.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5687,7 +5687,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart25.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5981,7 +5981,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart26.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6191,7 +6191,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart27.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6417,7 +6417,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart28.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6904,7 +6904,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -7436,7 +7436,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -7597,7 +7597,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8110,7 +8110,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8407,7 +8407,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8940,7 +8940,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:roundedCorners val="1"/>
   <c:chart>
     <c:title>
@@ -9459,7 +9459,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -9972,7 +9972,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -9997,67 +9997,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R82829a5de6ca470e"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame>
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="East Region Trend"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
-        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ac388eaeaf44e10"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame>
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="All Regions — Full Year"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
-        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R100cf27edf564e83"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a232e0d5cca44a8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10078,6 +10018,66 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="East Region Trend"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7d028fcae4594fc2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="All Regions — Full Year"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re9a7eab82ea94cc8"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="5" name="Simple Two-Series"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
@@ -10087,7 +10087,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R03c89398da534425"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7db34226703b4f29"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10097,7 +10097,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10122,7 +10122,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e7fc478db724364"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1a484f6974674d0a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10152,7 +10152,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R841ee3ecb7d0402e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec0dff9761ea4a1c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10160,15 +10160,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10182,7 +10182,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red44bd9154c24230"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb8887e528b654c1c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10212,7 +10212,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fd2c4af072545ff"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb54bf6adf35a4658"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10222,7 +10222,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10247,7 +10247,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R021cd8f727964d61"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c557bfe6b8b42b8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10277,7 +10277,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf4b57813c5db4e19"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05bf2db6710b453e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10287,13 +10287,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10307,7 +10307,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra1612f53fb1e4161"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8f5e35deb72498a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10337,7 +10337,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re94ae6bf33f4466a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb6864ace4f434fa7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10347,7 +10347,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10372,7 +10372,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R75aad71dea244387"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R713d04dadc424f16"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10402,7 +10402,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fa09b1ea30548bd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R34b9f1ebfc85406c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10432,7 +10432,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a1a02607934c97"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re2f4d66f4aed4411"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10462,7 +10462,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R949f5b039fb34a51"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R66ba99f7eec1447c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10472,7 +10472,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10497,7 +10497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06b22162442e48b6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf362b5e9910484d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10527,7 +10527,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabd58a4f2a184bad"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2dbb279b8e634812"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10557,7 +10557,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48ef8511e5a44b87"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R709b0fda82594d61"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10587,7 +10587,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0276fa5e078a45a5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9fd382b1e1b84731"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10597,7 +10597,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10622,7 +10622,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52d8ffb89eb74f4c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf63ba82354794c48"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10652,7 +10652,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc598170c9d43401b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R56a6d3312835445e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10682,7 +10682,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85863529710a43c3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R607c0fb91dda4b61"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10712,7 +10712,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0254af189de4690"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2e8e3c7da2224d3d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10722,7 +10722,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10747,7 +10747,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R84ee8024b2924161"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddf220fd100e4113"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10777,7 +10777,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R46f87f3b69aa4bf4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc2e4a043ce70430d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10807,7 +10807,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d936f56f57142d9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd46e119959794e2f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10837,7 +10837,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcd02a2c4cccc44b4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dec818039d84265"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -11075,50 +11075,50 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16f2ef06580438c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb700e86283954b52"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R622d87bf24db424a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1dc65648ad74637"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R274a82bc11674dff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bd62a4e93d54c83"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb2c7f1920614886"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe183d653c074707"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727c62ff98bc43b9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb58f90e02cb4068"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfee2e49219574a0b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R330f9cefc45e430e"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf044d4fd7a4014"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6214f4cac944f59"/>
 </x:worksheet>
 </file>
</xml_diff>